<commit_message>
add compatibility of train types
</commit_message>
<xml_diff>
--- a/Data/Base Day TUE.xlsx
+++ b/Data/Base Day TUE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meine Ablage\UNI\MSc DTU\Masterarbeit\RollingStock\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AFA7948-EDB5-4FAD-B66A-56F10225860C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44887652-818A-4CC8-8322-F4BCDDDAB171}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2730" yWindow="2730" windowWidth="21600" windowHeight="11295" tabRatio="819" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="819" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Manual" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="917" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="918" uniqueCount="326">
   <si>
     <t>Settings</t>
   </si>
@@ -1021,6 +1021,9 @@
   </si>
   <si>
     <t>Limitation on the number of units of equipment at the station at the end of the period</t>
+  </si>
+  <si>
+    <t>Electrified</t>
   </si>
 </sst>
 </file>
@@ -3546,7 +3549,7 @@
   <sheetPr codeName="Ark8">
     <tabColor theme="5" tint="0.59999389629810485"/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.28515625" customWidth="1"/>
@@ -3557,7 +3560,7 @@
     <col min="8" max="8" width="12.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>31</v>
       </c>
@@ -3582,8 +3585,11 @@
       <c r="H1" s="3" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1" s="3" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>203</v>
       </c>
@@ -3608,8 +3614,11 @@
       <c r="H2">
         <v>75</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>205</v>
       </c>
@@ -3634,8 +3643,11 @@
       <c r="H3">
         <v>37</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>105</v>
       </c>
@@ -3660,8 +3672,11 @@
       <c r="H4">
         <v>10</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>208</v>
       </c>
@@ -3686,8 +3701,11 @@
       <c r="H5">
         <v>10</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>210</v>
       </c>
@@ -3712,8 +3730,11 @@
       <c r="H6">
         <v>30</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>212</v>
       </c>
@@ -3738,8 +3759,11 @@
       <c r="H7">
         <v>4</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>260</v>
       </c>
@@ -3763,6 +3787,9 @@
       </c>
       <c r="H8">
         <v>7</v>
+      </c>
+      <c r="I8">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
base comp model is working
</commit_message>
<xml_diff>
--- a/Data/Base Day TUE.xlsx
+++ b/Data/Base Day TUE.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr codeName="Denne_projektmappe"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meine Ablage\UNI\MSc DTU\Masterarbeit\RollingStock\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44887652-818A-4CC8-8322-F4BCDDDAB171}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AFB6B02-701A-40D7-8700-3C3505CFF79A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="819" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="819" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Manual" sheetId="1" r:id="rId1"/>
@@ -45,6 +45,24 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={D5A09832-DCC1-4C14-988A-6790DFA22986}</author>
+  </authors>
+  <commentList>
+    <comment ref="A31" authorId="0" shapeId="0" xr:uid="{D5A09832-DCC1-4C14-988A-6790DFA22986}">
+      <text>
+        <t>[Kommentarthread]
+Ihre Version von Excel gestattet Ihnen das Lesen dieses Kommentarthreads. Jegliche Bearbeitungen daran werden jedoch entfernt, wenn die Datei in einer neueren Version von Excel geöffnet wird. Weitere Informationen: https://go.microsoft.com/fwlink/?linkid=870924.
+Kommentar:
+    There was a spelling mistake: it was Talco with a c before</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="918" uniqueCount="326">
   <si>
@@ -1033,7 +1051,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1064,6 +1082,12 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Segoe UI"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -1214,6 +1238,12 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Lukas Egkher" id="{C017F3F1-EF36-4905-B0C6-E2CF00B0F431}" userId="36c6e3171e52559e" providerId="Windows Live"/>
+</personList>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1477,6 +1507,14 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="A31" dT="2026-03-19T12:30:14.23" personId="{C017F3F1-EF36-4905-B0C6-E2CF00B0F431}" id="{D5A09832-DCC1-4C14-988A-6790DFA22986}">
+    <text>There was a spelling mistake: it was Talco with a c before</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Ark1">
@@ -3799,7 +3837,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <sheetPr codeName="Ark9">
     <tabColor theme="5" tint="0.59999389629810485"/>
   </sheetPr>
@@ -3964,7 +4002,7 @@
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>214</v>
+        <v>260</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
@@ -3993,6 +4031,7 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
change time format to integers for better processing add spelling mistake in BaseDayTUE
</commit_message>
<xml_diff>
--- a/Data/Base Day TUE.xlsx
+++ b/Data/Base Day TUE.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr codeName="Denne_projektmappe"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meine Ablage\UNI\MSc DTU\Masterarbeit\RollingStock\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44887652-818A-4CC8-8322-F4BCDDDAB171}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32221BC0-66DC-42E9-A382-EFDCC0874E63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="819" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="819" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Manual" sheetId="1" r:id="rId1"/>
@@ -3964,7 +3964,7 @@
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>214</v>
+        <v>260</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
composition model is running in around 600 seconds
</commit_message>
<xml_diff>
--- a/Data/Base Day TUE.xlsx
+++ b/Data/Base Day TUE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meine Ablage\UNI\MSc DTU\Masterarbeit\RollingStock\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31947851-F5AB-4655-BEA2-3DF92E0444B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{487B0154-1385-4975-BEB1-3DFAA753174D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="819" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="819" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Manual" sheetId="1" r:id="rId1"/>

</xml_diff>